<commit_message>
Added growing degree days (GDD5) to region parameters and min_GDD5 to crop parameters and implemented constraint C7 that limits cultivation of some crops in some regions based on minimum GDD
</commit_message>
<xml_diff>
--- a/data/prod_parameters/CropProduction.xlsx
+++ b/data/prod_parameters/CropProduction.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="209">
   <si>
     <t>f_crop</t>
   </si>
@@ -664,6 +664,27 @@
   </si>
   <si>
     <t>read from csv</t>
+  </si>
+  <si>
+    <t>min_GDD5</t>
+  </si>
+  <si>
+    <r>
+      <t>Minimum growing degree days</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Based on the number of growing degree days in the "coldest" region where the crop is currently (2016-2020) grown</t>
+    </r>
+  </si>
+  <si>
+    <t>C*days</t>
   </si>
 </sst>
 </file>
@@ -1852,7 +1873,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J139"/>
+  <dimension ref="A1:J196"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="30.42578125" customWidth="1"/>
@@ -3609,6 +3630,617 @@
       </c>
       <c r="I139" t="s">
         <v>205</v>
+      </c>
+    </row>
+    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A141" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B141" s="1"/>
+      <c r="C141" s="1"/>
+      <c r="D141" s="1"/>
+      <c r="E141" s="1"/>
+      <c r="F141" s="2"/>
+      <c r="G141" s="2"/>
+      <c r="H141" s="2"/>
+      <c r="I141" s="2"/>
+      <c r="J141" s="2"/>
+    </row>
+    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>10</v>
+      </c>
+      <c r="F143" t="s">
+        <v>206</v>
+      </c>
+      <c r="G143">
+        <v>1508</v>
+      </c>
+      <c r="H143" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>13</v>
+      </c>
+      <c r="F144" t="s">
+        <v>206</v>
+      </c>
+      <c r="G144">
+        <v>980</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>14</v>
+      </c>
+      <c r="F145" t="s">
+        <v>206</v>
+      </c>
+      <c r="G145">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>154</v>
+      </c>
+      <c r="F146" t="s">
+        <v>206</v>
+      </c>
+      <c r="G146">
+        <v>1779</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>15</v>
+      </c>
+      <c r="F147" t="s">
+        <v>206</v>
+      </c>
+      <c r="G147">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>16</v>
+      </c>
+      <c r="F148" t="s">
+        <v>206</v>
+      </c>
+      <c r="G148">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>110</v>
+      </c>
+      <c r="F149" t="s">
+        <v>206</v>
+      </c>
+      <c r="G149">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>17</v>
+      </c>
+      <c r="F150" t="s">
+        <v>206</v>
+      </c>
+      <c r="G150">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>111</v>
+      </c>
+      <c r="F151" t="s">
+        <v>206</v>
+      </c>
+      <c r="G151">
+        <v>1185</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>160</v>
+      </c>
+      <c r="F152" t="s">
+        <v>206</v>
+      </c>
+      <c r="G152">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>112</v>
+      </c>
+      <c r="F153" t="s">
+        <v>206</v>
+      </c>
+      <c r="G153">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>113</v>
+      </c>
+      <c r="F154" t="s">
+        <v>206</v>
+      </c>
+      <c r="G154">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>18</v>
+      </c>
+      <c r="F155" t="s">
+        <v>206</v>
+      </c>
+      <c r="G155">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>19</v>
+      </c>
+      <c r="F156" t="s">
+        <v>206</v>
+      </c>
+      <c r="G156">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>20</v>
+      </c>
+      <c r="F157" t="s">
+        <v>206</v>
+      </c>
+      <c r="G157">
+        <v>1185</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>114</v>
+      </c>
+      <c r="F158" t="s">
+        <v>206</v>
+      </c>
+      <c r="G158">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>21</v>
+      </c>
+      <c r="F159" t="s">
+        <v>206</v>
+      </c>
+      <c r="G159">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>115</v>
+      </c>
+      <c r="F160" t="s">
+        <v>206</v>
+      </c>
+      <c r="G160">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>22</v>
+      </c>
+      <c r="F161" t="s">
+        <v>206</v>
+      </c>
+      <c r="G161">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>23</v>
+      </c>
+      <c r="F162" t="s">
+        <v>206</v>
+      </c>
+      <c r="G162">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>24</v>
+      </c>
+      <c r="F163" t="s">
+        <v>206</v>
+      </c>
+      <c r="G163">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>116</v>
+      </c>
+      <c r="F164" t="s">
+        <v>206</v>
+      </c>
+      <c r="G164">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>25</v>
+      </c>
+      <c r="F165" t="s">
+        <v>206</v>
+      </c>
+      <c r="G165">
+        <v>1487</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>26</v>
+      </c>
+      <c r="F166" t="s">
+        <v>206</v>
+      </c>
+      <c r="G166">
+        <v>1487</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>117</v>
+      </c>
+      <c r="F167" t="s">
+        <v>206</v>
+      </c>
+      <c r="G167">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>27</v>
+      </c>
+      <c r="F168" t="s">
+        <v>206</v>
+      </c>
+      <c r="G168">
+        <v>980</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>118</v>
+      </c>
+      <c r="F169" t="s">
+        <v>206</v>
+      </c>
+      <c r="G169">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>28</v>
+      </c>
+      <c r="F170" t="s">
+        <v>206</v>
+      </c>
+      <c r="G170">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>119</v>
+      </c>
+      <c r="F171" t="s">
+        <v>206</v>
+      </c>
+      <c r="G171">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>29</v>
+      </c>
+      <c r="F172" t="s">
+        <v>206</v>
+      </c>
+      <c r="G172">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>30</v>
+      </c>
+      <c r="F173" t="s">
+        <v>206</v>
+      </c>
+      <c r="G173">
+        <v>1508</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>120</v>
+      </c>
+      <c r="F174" t="s">
+        <v>206</v>
+      </c>
+      <c r="G174">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>31</v>
+      </c>
+      <c r="F175" t="s">
+        <v>206</v>
+      </c>
+      <c r="G175">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>121</v>
+      </c>
+      <c r="F176" t="s">
+        <v>206</v>
+      </c>
+      <c r="G176">
+        <v>1185</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>122</v>
+      </c>
+      <c r="F177" t="s">
+        <v>206</v>
+      </c>
+      <c r="G177">
+        <v>1508</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>32</v>
+      </c>
+      <c r="F178" t="s">
+        <v>206</v>
+      </c>
+      <c r="G178">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>33</v>
+      </c>
+      <c r="F179" t="s">
+        <v>206</v>
+      </c>
+      <c r="G179">
+        <v>1569</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>123</v>
+      </c>
+      <c r="F180" t="s">
+        <v>206</v>
+      </c>
+      <c r="G180">
+        <v>1569</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>124</v>
+      </c>
+      <c r="F181" t="s">
+        <v>206</v>
+      </c>
+      <c r="G181">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>125</v>
+      </c>
+      <c r="F182" t="s">
+        <v>206</v>
+      </c>
+      <c r="G182">
+        <v>1185</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>126</v>
+      </c>
+      <c r="F183" t="s">
+        <v>206</v>
+      </c>
+      <c r="G183">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>127</v>
+      </c>
+      <c r="F184" t="s">
+        <v>206</v>
+      </c>
+      <c r="G184">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>35</v>
+      </c>
+      <c r="F185" t="s">
+        <v>206</v>
+      </c>
+      <c r="G185">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>36</v>
+      </c>
+      <c r="F186" t="s">
+        <v>206</v>
+      </c>
+      <c r="G186">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>37</v>
+      </c>
+      <c r="F187" t="s">
+        <v>206</v>
+      </c>
+      <c r="G187">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>128</v>
+      </c>
+      <c r="F188" t="s">
+        <v>206</v>
+      </c>
+      <c r="G188">
+        <v>1225</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>38</v>
+      </c>
+      <c r="F189" t="s">
+        <v>206</v>
+      </c>
+      <c r="G189">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>129</v>
+      </c>
+      <c r="F190" t="s">
+        <v>206</v>
+      </c>
+      <c r="G190">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>39</v>
+      </c>
+      <c r="F191" t="s">
+        <v>206</v>
+      </c>
+      <c r="G191">
+        <v>1721</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>130</v>
+      </c>
+      <c r="F192" t="s">
+        <v>206</v>
+      </c>
+      <c r="G192">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>40</v>
+      </c>
+      <c r="F193" t="s">
+        <v>206</v>
+      </c>
+      <c r="G193">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>41</v>
+      </c>
+      <c r="F194" t="s">
+        <v>206</v>
+      </c>
+      <c r="G194">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>42</v>
+      </c>
+      <c r="F195" t="s">
+        <v>206</v>
+      </c>
+      <c r="G195">
+        <v>980</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>43</v>
+      </c>
+      <c r="F196" t="s">
+        <v>206</v>
+      </c>
+      <c r="G196">
+        <v>1016</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix crop_to_prod 'Mixed cereals'
</commit_message>
<xml_diff>
--- a/data/prod_parameters/CropProduction.xlsx
+++ b/data/prod_parameters/CropProduction.xlsx
@@ -2085,7 +2085,7 @@
         <v>53</v>
       </c>
       <c r="G13" s="4">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -2099,7 +2099,7 @@
         <v>53</v>
       </c>
       <c r="G14" s="4">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Implemented method for VS excretion and losses
</commit_message>
<xml_diff>
--- a/data/prod_parameters/CropProduction.xlsx
+++ b/data/prod_parameters/CropProduction.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="239">
   <si>
     <t>f_crop</t>
   </si>
@@ -760,6 +760,21 @@
   </si>
   <si>
     <t>CropProduction-yields.csv</t>
+  </si>
+  <si>
+    <t>kg DM</t>
+  </si>
+  <si>
+    <t>kg @ 14% w.c.</t>
+  </si>
+  <si>
+    <t>Anta potentiell skörd</t>
+  </si>
+  <si>
+    <t>Skörd från Pierre</t>
+  </si>
+  <si>
+    <t>Anta skörd utifrån vall?</t>
   </si>
 </sst>
 </file>
@@ -2029,6 +2044,9 @@
       <c r="F4">
         <v>1</v>
       </c>
+      <c r="G4" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -2201,7 +2219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -2215,7 +2233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>152</v>
       </c>
@@ -2229,7 +2247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>125</v>
       </c>
@@ -2243,7 +2261,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>124</v>
       </c>
@@ -2257,7 +2275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>122</v>
       </c>
@@ -2271,7 +2289,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>121</v>
       </c>
@@ -2285,7 +2303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>39</v>
       </c>
@@ -2299,7 +2317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -2313,7 +2331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2327,8 +2345,11 @@
       <c r="F25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G25" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>23</v>
       </c>
@@ -2342,8 +2363,11 @@
       <c r="F26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G26" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>26</v>
       </c>
@@ -2357,8 +2381,11 @@
       <c r="F27">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G27" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>17</v>
       </c>
@@ -2372,8 +2399,11 @@
       <c r="F28">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G28" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>29</v>
       </c>
@@ -2387,8 +2417,11 @@
       <c r="F29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G29" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>37</v>
       </c>
@@ -2402,8 +2435,11 @@
       <c r="F30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G30" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>36</v>
       </c>
@@ -2417,8 +2453,11 @@
       <c r="F31">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G31" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>116</v>
       </c>
@@ -2741,36 +2780,61 @@
       <c r="A56" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B56" s="4"/>
-      <c r="F56" s="4"/>
+      <c r="B56" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E56" t="s">
+        <v>51</v>
+      </c>
+      <c r="F56" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B57" s="4"/>
-      <c r="F57" s="4"/>
+      <c r="B57" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="F57" s="10"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B58" s="4"/>
-      <c r="F58" s="4"/>
+      <c r="B58" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="F58" s="10"/>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B59" s="4"/>
-      <c r="F59" s="4"/>
+      <c r="B59" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E59" t="s">
+        <v>51</v>
+      </c>
+      <c r="F59" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B60" s="4"/>
-      <c r="F60" s="4"/>
+      <c r="B60" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E60" t="s">
+        <v>51</v>
+      </c>
+      <c r="F60" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="4"/>

</xml_diff>

<commit_message>
First stab at calculating C in manure + function to transfer data to ICBM for soil carbon calculation
</commit_message>
<xml_diff>
--- a/data/prod_parameters/CropProduction.xlsx
+++ b/data/prod_parameters/CropProduction.xlsx
@@ -4,13 +4,11 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="11520" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="11520"/>
   </bookViews>
   <sheets>
-    <sheet name="description" sheetId="2" r:id="rId1"/>
-    <sheet name="relations" sheetId="4" r:id="rId2"/>
-    <sheet name="default" sheetId="1" r:id="rId3"/>
-    <sheet name="scn_baseline" sheetId="3" r:id="rId4"/>
+    <sheet name="default" sheetId="1" r:id="rId1"/>
+    <sheet name="references" sheetId="5" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -22,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="170">
   <si>
     <t>f_crop</t>
   </si>
@@ -126,9 +124,6 @@
     <t>Peas, green</t>
   </si>
   <si>
-    <t>Potatoes</t>
-  </si>
-  <si>
     <t>Rye</t>
   </si>
   <si>
@@ -162,204 +157,21 @@
     <t>wheat</t>
   </si>
   <si>
-    <r>
-      <t>Yields</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (parameter = yield)</t>
-    </r>
-  </si>
-  <si>
     <t>maize fodder</t>
   </si>
   <si>
-    <t>y_2020</t>
-  </si>
-  <si>
-    <t>y_2050</t>
-  </si>
-  <si>
     <t>grazing</t>
   </si>
   <si>
     <t>crop_to_prod</t>
   </si>
   <si>
-    <t>crop</t>
-  </si>
-  <si>
-    <t>crop_group</t>
-  </si>
-  <si>
-    <t>land_use</t>
-  </si>
-  <si>
-    <t>cropland</t>
-  </si>
-  <si>
     <t>Grain legumes</t>
   </si>
   <si>
     <t>Brassicaceae</t>
   </si>
   <si>
-    <t>Beets</t>
-  </si>
-  <si>
-    <t>Berries</t>
-  </si>
-  <si>
-    <t>Fruit trees</t>
-  </si>
-  <si>
-    <t>Vegetables</t>
-  </si>
-  <si>
-    <t>Fodder crops</t>
-  </si>
-  <si>
-    <t>Ley</t>
-  </si>
-  <si>
-    <t>Energy crops</t>
-  </si>
-  <si>
-    <t>Cereals, winter</t>
-  </si>
-  <si>
-    <t>Cereals, spring</t>
-  </si>
-  <si>
-    <t>CPC</t>
-  </si>
-  <si>
-    <t>0111.S</t>
-  </si>
-  <si>
-    <t>0111.W</t>
-  </si>
-  <si>
-    <t>0112</t>
-  </si>
-  <si>
-    <t>0115.S</t>
-  </si>
-  <si>
-    <t>0115.W</t>
-  </si>
-  <si>
-    <t>0116</t>
-  </si>
-  <si>
-    <t>0117</t>
-  </si>
-  <si>
-    <t>01191.S</t>
-  </si>
-  <si>
-    <t>01191.W</t>
-  </si>
-  <si>
-    <t>01199.02</t>
-  </si>
-  <si>
-    <t>012.O</t>
-  </si>
-  <si>
-    <t>0121.C</t>
-  </si>
-  <si>
-    <t>0121.H</t>
-  </si>
-  <si>
-    <t>0121.L</t>
-  </si>
-  <si>
-    <t>01232</t>
-  </si>
-  <si>
-    <t>01235</t>
-  </si>
-  <si>
-    <t>01242</t>
-  </si>
-  <si>
-    <t>01251</t>
-  </si>
-  <si>
-    <t>01259</t>
-  </si>
-  <si>
-    <t>0134.O</t>
-  </si>
-  <si>
-    <t>01341</t>
-  </si>
-  <si>
-    <t>0135.O</t>
-  </si>
-  <si>
-    <t>01354</t>
-  </si>
-  <si>
-    <t>01443.S</t>
-  </si>
-  <si>
-    <t>01443.W</t>
-  </si>
-  <si>
-    <t>01701</t>
-  </si>
-  <si>
-    <t>01702</t>
-  </si>
-  <si>
-    <t>01705</t>
-  </si>
-  <si>
-    <t>01801</t>
-  </si>
-  <si>
-    <t>01911</t>
-  </si>
-  <si>
-    <t>01919.C</t>
-  </si>
-  <si>
-    <t>01919.FAL</t>
-  </si>
-  <si>
-    <t>01919.GM</t>
-  </si>
-  <si>
-    <t>01919.L.F</t>
-  </si>
-  <si>
-    <t>01919.L.G</t>
-  </si>
-  <si>
-    <t>01919.L.S</t>
-  </si>
-  <si>
-    <t>01919.O</t>
-  </si>
-  <si>
-    <t>01919.SNG.F</t>
-  </si>
-  <si>
-    <t>01919.SNG.G</t>
-  </si>
-  <si>
-    <t>kg DM or WW/ha or m2 (depending on crop)</t>
-  </si>
-  <si>
     <t>Carrots</t>
   </si>
   <si>
@@ -421,66 +233,6 @@
   </si>
   <si>
     <t>Tomatoes, greenhouse</t>
-  </si>
-  <si>
-    <t>01510.T</t>
-  </si>
-  <si>
-    <t>01510.S</t>
-  </si>
-  <si>
-    <t>0199.EG</t>
-  </si>
-  <si>
-    <t>0199.SRC</t>
-  </si>
-  <si>
-    <t>01919.L.NH</t>
-  </si>
-  <si>
-    <t>Semi-natural grasslands</t>
-  </si>
-  <si>
-    <t>semi-natural grasslands</t>
-  </si>
-  <si>
-    <t>01253</t>
-  </si>
-  <si>
-    <t>01351</t>
-  </si>
-  <si>
-    <t>01342</t>
-  </si>
-  <si>
-    <t>01234.GH</t>
-  </si>
-  <si>
-    <t>01232.GH</t>
-  </si>
-  <si>
-    <t>01214.GH</t>
-  </si>
-  <si>
-    <t>012.O.GH</t>
-  </si>
-  <si>
-    <t>0121.H.GH</t>
-  </si>
-  <si>
-    <t>01354.GH</t>
-  </si>
-  <si>
-    <t>0135.O.GH</t>
-  </si>
-  <si>
-    <t>Vegetables, greenhouse</t>
-  </si>
-  <si>
-    <t>Berries, greenhouse</t>
-  </si>
-  <si>
-    <t>greenhouse</t>
   </si>
   <si>
     <r>
@@ -675,9 +427,6 @@
     </r>
   </si>
   <si>
-    <t>C*days</t>
-  </si>
-  <si>
     <t>ag_resid</t>
   </si>
   <si>
@@ -765,9 +514,6 @@
     <t>kg DM</t>
   </si>
   <si>
-    <t>kg @ 14% w.c.</t>
-  </si>
-  <si>
     <t>Anta potentiell skörd</t>
   </si>
   <si>
@@ -775,6 +521,39 @@
   </si>
   <si>
     <t>Anta skörd utifrån vall?</t>
+  </si>
+  <si>
+    <t>kg @ 86% DM</t>
+  </si>
+  <si>
+    <t>kg @ 85% DM</t>
+  </si>
+  <si>
+    <t>NIR 2022; Jacobs et al 2020</t>
+  </si>
+  <si>
+    <t>Jacobs, A., Poeplau, C., Weiser, C., Fahrion-Nitschke, A., &amp; Don, A. (2020). Exports and inputs of organic carbon on agricultural soils in Germany. Nutrient Cycling in Agroecosystems, 118(3), 249-271. doi:10.1007/s10705-020-10087-5</t>
+  </si>
+  <si>
+    <t>NIR (2022) National Inventory Report Sweden 2022 - Greenhouse Gas Emission Inventories 1990-2020. Swedish Environmental Protection Agency</t>
+  </si>
+  <si>
+    <t>NIR 2022</t>
+  </si>
+  <si>
+    <t>No seeding</t>
+  </si>
+  <si>
+    <t>kg/m2</t>
+  </si>
+  <si>
+    <t>kg DM or w.w. / ha (or m2 for greenhouse crops)</t>
+  </si>
+  <si>
+    <t>C(&gt;5C)*days (??)</t>
+  </si>
+  <si>
+    <t>Yields</t>
   </si>
 </sst>
 </file>
@@ -784,7 +563,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -810,14 +589,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -871,21 +642,20 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
@@ -1169,801 +939,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="44.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.42578125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" t="s">
-        <v>65</v>
-      </c>
-      <c r="D5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D6" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>74</v>
-      </c>
-      <c r="B7" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>76</v>
-      </c>
-      <c r="B8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" t="s">
-        <v>65</v>
-      </c>
-      <c r="D8" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>75</v>
-      </c>
-      <c r="B9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" t="s">
-        <v>66</v>
-      </c>
-      <c r="D9" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>70</v>
-      </c>
-      <c r="B10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" t="s">
-        <v>66</v>
-      </c>
-      <c r="D10" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>77</v>
-      </c>
-      <c r="B11" t="s">
-        <v>115</v>
-      </c>
-      <c r="C11" t="s">
-        <v>66</v>
-      </c>
-      <c r="D11" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>95</v>
-      </c>
-      <c r="B12" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D12" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>84</v>
-      </c>
-      <c r="B13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C13" t="s">
-        <v>56</v>
-      </c>
-      <c r="D13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>94</v>
-      </c>
-      <c r="B14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" t="s">
-        <v>56</v>
-      </c>
-      <c r="D14" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>93</v>
-      </c>
-      <c r="B15" t="s">
-        <v>152</v>
-      </c>
-      <c r="C15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D15" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>92</v>
-      </c>
-      <c r="B16" t="s">
-        <v>125</v>
-      </c>
-      <c r="C16" t="s">
-        <v>57</v>
-      </c>
-      <c r="D16" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>91</v>
-      </c>
-      <c r="B17" t="s">
-        <v>124</v>
-      </c>
-      <c r="C17" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>129</v>
-      </c>
-      <c r="B18" t="s">
-        <v>122</v>
-      </c>
-      <c r="C18" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>130</v>
-      </c>
-      <c r="B19" t="s">
-        <v>121</v>
-      </c>
-      <c r="C19" t="s">
-        <v>34</v>
-      </c>
-      <c r="D19" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>96</v>
-      </c>
-      <c r="B20" t="s">
-        <v>39</v>
-      </c>
-      <c r="C20" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>103</v>
-      </c>
-      <c r="B21" t="s">
-        <v>24</v>
-      </c>
-      <c r="C21" t="s">
-        <v>63</v>
-      </c>
-      <c r="D21" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>99</v>
-      </c>
-      <c r="B22" t="s">
-        <v>18</v>
-      </c>
-      <c r="C22" t="s">
-        <v>18</v>
-      </c>
-      <c r="D22" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>131</v>
-      </c>
-      <c r="B23" t="s">
-        <v>111</v>
-      </c>
-      <c r="C23" t="s">
-        <v>64</v>
-      </c>
-      <c r="D23" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>132</v>
-      </c>
-      <c r="B24" t="s">
-        <v>126</v>
-      </c>
-      <c r="C24" t="s">
-        <v>64</v>
-      </c>
-      <c r="D24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>100</v>
-      </c>
-      <c r="B25" t="s">
-        <v>19</v>
-      </c>
-      <c r="C25" t="s">
-        <v>19</v>
-      </c>
-      <c r="D25" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>101</v>
-      </c>
-      <c r="B26" t="s">
-        <v>22</v>
-      </c>
-      <c r="C26" t="s">
-        <v>63</v>
-      </c>
-      <c r="D26" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>102</v>
-      </c>
-      <c r="B27" t="s">
-        <v>23</v>
-      </c>
-      <c r="C27" t="s">
-        <v>63</v>
-      </c>
-      <c r="D27" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>133</v>
-      </c>
-      <c r="B28" t="s">
-        <v>114</v>
-      </c>
-      <c r="C28" t="s">
-        <v>63</v>
-      </c>
-      <c r="D28" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>97</v>
-      </c>
-      <c r="B29" t="s">
-        <v>26</v>
-      </c>
-      <c r="C29" t="s">
-        <v>62</v>
-      </c>
-      <c r="D29" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>98</v>
-      </c>
-      <c r="B30" t="s">
-        <v>17</v>
-      </c>
-      <c r="C30" t="s">
-        <v>62</v>
-      </c>
-      <c r="D30" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>104</v>
-      </c>
-      <c r="B31" t="s">
-        <v>29</v>
-      </c>
-      <c r="C31" t="s">
-        <v>62</v>
-      </c>
-      <c r="D31" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>106</v>
-      </c>
-      <c r="B32" t="s">
-        <v>37</v>
-      </c>
-      <c r="C32" t="s">
-        <v>134</v>
-      </c>
-      <c r="D32" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>105</v>
-      </c>
-      <c r="B33" t="s">
-        <v>36</v>
-      </c>
-      <c r="C33" t="s">
-        <v>134</v>
-      </c>
-      <c r="D33" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>136</v>
-      </c>
-      <c r="B34" t="s">
-        <v>116</v>
-      </c>
-      <c r="C34" t="s">
-        <v>61</v>
-      </c>
-      <c r="D34" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>85</v>
-      </c>
-      <c r="B35" t="s">
-        <v>108</v>
-      </c>
-      <c r="C35" t="s">
-        <v>61</v>
-      </c>
-      <c r="D35" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>86</v>
-      </c>
-      <c r="B36" t="s">
-        <v>118</v>
-      </c>
-      <c r="C36" t="s">
-        <v>61</v>
-      </c>
-      <c r="D36" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>81</v>
-      </c>
-      <c r="B37" t="s">
-        <v>21</v>
-      </c>
-      <c r="C37" t="s">
-        <v>61</v>
-      </c>
-      <c r="D37" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>79</v>
-      </c>
-      <c r="B38" t="s">
-        <v>16</v>
-      </c>
-      <c r="C38" t="s">
-        <v>61</v>
-      </c>
-      <c r="D38" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>82</v>
-      </c>
-      <c r="B39" t="s">
-        <v>109</v>
-      </c>
-      <c r="C39" t="s">
-        <v>61</v>
-      </c>
-      <c r="D39" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>83</v>
-      </c>
-      <c r="B40" t="s">
-        <v>123</v>
-      </c>
-      <c r="C40" t="s">
-        <v>61</v>
-      </c>
-      <c r="D40" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>80</v>
-      </c>
-      <c r="B41" t="s">
-        <v>20</v>
-      </c>
-      <c r="C41" t="s">
-        <v>61</v>
-      </c>
-      <c r="D41" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>78</v>
-      </c>
-      <c r="B42" t="s">
-        <v>31</v>
-      </c>
-      <c r="C42" t="s">
-        <v>61</v>
-      </c>
-      <c r="D42" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>90</v>
-      </c>
-      <c r="B43" t="s">
-        <v>38</v>
-      </c>
-      <c r="C43" t="s">
-        <v>59</v>
-      </c>
-      <c r="D43" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>137</v>
-      </c>
-      <c r="B44" t="s">
-        <v>110</v>
-      </c>
-      <c r="C44" t="s">
-        <v>59</v>
-      </c>
-      <c r="D44" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>89</v>
-      </c>
-      <c r="B45" t="s">
-        <v>28</v>
-      </c>
-      <c r="C45" t="s">
-        <v>59</v>
-      </c>
-      <c r="D45" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>88</v>
-      </c>
-      <c r="B46" t="s">
-        <v>10</v>
-      </c>
-      <c r="C46" t="s">
-        <v>60</v>
-      </c>
-      <c r="D46" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>138</v>
-      </c>
-      <c r="B47" t="s">
-        <v>120</v>
-      </c>
-      <c r="C47" t="s">
-        <v>60</v>
-      </c>
-      <c r="D47" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>87</v>
-      </c>
-      <c r="B48" t="s">
-        <v>30</v>
-      </c>
-      <c r="C48" t="s">
-        <v>60</v>
-      </c>
-      <c r="D48" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>139</v>
-      </c>
-      <c r="B49" t="s">
-        <v>128</v>
-      </c>
-      <c r="C49" t="s">
-        <v>146</v>
-      </c>
-      <c r="D49" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>140</v>
-      </c>
-      <c r="B50" t="s">
-        <v>158</v>
-      </c>
-      <c r="C50" t="s">
-        <v>146</v>
-      </c>
-      <c r="D50" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>141</v>
-      </c>
-      <c r="B51" t="s">
-        <v>113</v>
-      </c>
-      <c r="C51" t="s">
-        <v>146</v>
-      </c>
-      <c r="D51" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>142</v>
-      </c>
-      <c r="B52" t="s">
-        <v>119</v>
-      </c>
-      <c r="C52" t="s">
-        <v>146</v>
-      </c>
-      <c r="D52" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>143</v>
-      </c>
-      <c r="B53" t="s">
-        <v>112</v>
-      </c>
-      <c r="C53" t="s">
-        <v>146</v>
-      </c>
-      <c r="D53" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>144</v>
-      </c>
-      <c r="B54" t="s">
-        <v>127</v>
-      </c>
-      <c r="C54" t="s">
-        <v>147</v>
-      </c>
-      <c r="D54" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>145</v>
-      </c>
-      <c r="B55" t="s">
-        <v>117</v>
-      </c>
-      <c r="C55" t="s">
-        <v>147</v>
-      </c>
-      <c r="D55" t="s">
-        <v>148</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I215"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1982,7 +957,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>199</v>
+        <v>121</v>
       </c>
       <c r="C1" t="s">
         <v>9</v>
@@ -2008,7 +983,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>149</v>
+        <v>71</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2020,61 +995,67 @@
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E3" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="F3" s="6">
+      <c r="E3" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="5">
         <v>0</v>
       </c>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6" t="s">
-        <v>151</v>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>235</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B5" s="3"/>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F5">
         <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>153</v>
+        <v>75</v>
       </c>
       <c r="E6" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F6">
         <v>1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -2083,13 +1064,16 @@
       </c>
       <c r="B7" s="3"/>
       <c r="D7" t="s">
-        <v>150</v>
+        <v>72</v>
       </c>
       <c r="E7" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F7">
         <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -2098,13 +1082,16 @@
       </c>
       <c r="B8" s="3"/>
       <c r="D8" t="s">
-        <v>150</v>
+        <v>72</v>
       </c>
       <c r="E8" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F8">
         <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -2112,41 +1099,50 @@
         <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>154</v>
+        <v>76</v>
       </c>
       <c r="E9" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F9">
         <v>1</v>
+      </c>
+      <c r="G9" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>161</v>
+        <v>83</v>
       </c>
       <c r="E10" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F10">
         <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D11" t="s">
-        <v>161</v>
+        <v>83</v>
       </c>
       <c r="E11" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F11">
         <v>1</v>
+      </c>
+      <c r="G11" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -2154,41 +1150,50 @@
         <v>25</v>
       </c>
       <c r="D12" t="s">
-        <v>170</v>
+        <v>92</v>
       </c>
       <c r="E12" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F12">
         <v>1</v>
+      </c>
+      <c r="G12" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>115</v>
+        <v>57</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>162</v>
+        <v>84</v>
       </c>
       <c r="E13" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F13" s="4">
         <v>0.2</v>
       </c>
+      <c r="G13" s="4" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>115</v>
+        <v>57</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>154</v>
+        <v>76</v>
       </c>
       <c r="E14" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F14" s="4">
         <v>0.8</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -2196,27 +1201,33 @@
         <v>32</v>
       </c>
       <c r="D15" t="s">
-        <v>162</v>
+        <v>84</v>
       </c>
       <c r="E15" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F15">
         <v>1</v>
+      </c>
+      <c r="G15" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>33</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>169</v>
+      <c r="D16" s="6" t="s">
+        <v>91</v>
       </c>
       <c r="E16" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F16">
         <v>1</v>
+      </c>
+      <c r="G16" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2224,24 +1235,27 @@
         <v>15</v>
       </c>
       <c r="D17" t="s">
-        <v>163</v>
+        <v>85</v>
       </c>
       <c r="E17" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F17">
         <v>1</v>
+      </c>
+      <c r="G17" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>152</v>
+        <v>74</v>
       </c>
       <c r="D18" t="s">
-        <v>171</v>
+        <v>93</v>
       </c>
       <c r="E18" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F18">
         <v>1</v>
@@ -2249,13 +1263,13 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>125</v>
+        <v>67</v>
       </c>
       <c r="D19" t="s">
-        <v>160</v>
+        <v>82</v>
       </c>
       <c r="E19" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F19">
         <v>1</v>
@@ -2263,13 +1277,13 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>124</v>
+        <v>66</v>
       </c>
       <c r="D20" t="s">
-        <v>160</v>
+        <v>82</v>
       </c>
       <c r="E20" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -2277,13 +1291,13 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>122</v>
+        <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>156</v>
+        <v>78</v>
       </c>
       <c r="E21" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F21">
         <v>1</v>
@@ -2291,13 +1305,13 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>121</v>
+        <v>63</v>
       </c>
       <c r="D22" t="s">
-        <v>155</v>
+        <v>77</v>
       </c>
       <c r="E22" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F22">
         <v>1</v>
@@ -2305,13 +1319,13 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D23" t="s">
-        <v>172</v>
+        <v>94</v>
       </c>
       <c r="E23" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F23">
         <v>1</v>
@@ -2322,10 +1336,10 @@
         <v>24</v>
       </c>
       <c r="D24" t="s">
-        <v>173</v>
+        <v>95</v>
       </c>
       <c r="E24" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F24">
         <v>1</v>
@@ -2337,16 +1351,16 @@
       </c>
       <c r="B25" s="3"/>
       <c r="D25" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E25" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F25">
         <v>1</v>
       </c>
       <c r="G25" t="s">
-        <v>234</v>
+        <v>155</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -2355,16 +1369,16 @@
       </c>
       <c r="B26" s="3"/>
       <c r="D26" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E26" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F26">
         <v>1</v>
       </c>
       <c r="G26" t="s">
-        <v>234</v>
+        <v>155</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -2373,16 +1387,16 @@
       </c>
       <c r="B27" s="3"/>
       <c r="D27" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E27" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F27">
         <v>1</v>
       </c>
       <c r="G27" t="s">
-        <v>234</v>
+        <v>155</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -2391,16 +1405,16 @@
       </c>
       <c r="B28" s="3"/>
       <c r="D28" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E28" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F28">
         <v>1</v>
       </c>
       <c r="G28" t="s">
-        <v>234</v>
+        <v>155</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -2409,63 +1423,63 @@
       </c>
       <c r="B29" s="3"/>
       <c r="D29" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E29" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F29">
         <v>1</v>
       </c>
       <c r="G29" t="s">
-        <v>234</v>
+        <v>155</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B30" s="3"/>
       <c r="D30" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E30" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F30">
         <v>1</v>
       </c>
       <c r="G30" t="s">
-        <v>234</v>
+        <v>155</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B31" s="3"/>
       <c r="D31" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E31" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F31">
         <v>1</v>
       </c>
       <c r="G31" t="s">
-        <v>234</v>
+        <v>155</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>116</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>165</v>
+        <v>58</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>87</v>
       </c>
       <c r="E32" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -2473,13 +1487,13 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>108</v>
+        <v>50</v>
       </c>
       <c r="D33" t="s">
-        <v>164</v>
+        <v>86</v>
       </c>
       <c r="E33" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F33">
         <v>1</v>
@@ -2487,14 +1501,14 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>118</v>
+        <v>60</v>
       </c>
       <c r="B34" s="4"/>
       <c r="D34" s="4" t="s">
-        <v>164</v>
+        <v>86</v>
       </c>
       <c r="E34" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F34">
         <v>1</v>
@@ -2504,11 +1518,11 @@
       <c r="A35" t="s">
         <v>21</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>167</v>
+      <c r="D35" s="6" t="s">
+        <v>89</v>
       </c>
       <c r="E35" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F35">
         <v>1</v>
@@ -2518,11 +1532,11 @@
       <c r="A36" t="s">
         <v>16</v>
       </c>
-      <c r="D36" s="7" t="s">
-        <v>166</v>
+      <c r="D36" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="E36" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F36">
         <v>1</v>
@@ -2530,13 +1544,13 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>109</v>
+        <v>51</v>
       </c>
       <c r="D37" t="s">
-        <v>159</v>
+        <v>81</v>
       </c>
       <c r="E37" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F37">
         <v>1</v>
@@ -2544,13 +1558,13 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>123</v>
-      </c>
-      <c r="D38" s="7" t="s">
-        <v>168</v>
+        <v>65</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>90</v>
       </c>
       <c r="E38" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F38">
         <v>1</v>
@@ -2561,11 +1575,11 @@
         <v>20</v>
       </c>
       <c r="B39" s="4"/>
-      <c r="D39" s="8" t="s">
-        <v>182</v>
+      <c r="D39" s="7" t="s">
+        <v>104</v>
       </c>
       <c r="E39" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F39">
         <v>1</v>
@@ -2576,11 +1590,11 @@
         <v>31</v>
       </c>
       <c r="B40" s="4"/>
-      <c r="D40" s="8" t="s">
-        <v>179</v>
+      <c r="D40" s="7" t="s">
+        <v>101</v>
       </c>
       <c r="E40" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F40">
         <v>1</v>
@@ -2588,13 +1602,13 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>38</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>175</v>
+        <v>37</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>97</v>
       </c>
       <c r="E41" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -2602,13 +1616,13 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>110</v>
-      </c>
-      <c r="D42" s="7" t="s">
-        <v>178</v>
+        <v>52</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>100</v>
       </c>
       <c r="E42" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F42">
         <v>1</v>
@@ -2618,11 +1632,11 @@
       <c r="A43" t="s">
         <v>28</v>
       </c>
-      <c r="D43" s="7" t="s">
-        <v>181</v>
+      <c r="D43" s="6" t="s">
+        <v>103</v>
       </c>
       <c r="E43" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -2632,11 +1646,11 @@
       <c r="A44" t="s">
         <v>10</v>
       </c>
-      <c r="D44" s="7" t="s">
-        <v>176</v>
+      <c r="D44" s="6" t="s">
+        <v>98</v>
       </c>
       <c r="E44" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F44">
         <v>1</v>
@@ -2644,13 +1658,13 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>120</v>
-      </c>
-      <c r="D45" s="7" t="s">
-        <v>177</v>
+        <v>62</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>99</v>
       </c>
       <c r="E45" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F45">
         <v>1</v>
@@ -2660,11 +1674,11 @@
       <c r="A46" t="s">
         <v>30</v>
       </c>
-      <c r="D46" s="7" t="s">
-        <v>180</v>
+      <c r="D46" s="6" t="s">
+        <v>102</v>
       </c>
       <c r="E46" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F46">
         <v>1</v>
@@ -2672,13 +1686,13 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="D47" t="s">
-        <v>157</v>
+        <v>79</v>
       </c>
       <c r="E47" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F47">
         <v>1</v>
@@ -2686,13 +1700,13 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>158</v>
+        <v>80</v>
       </c>
       <c r="D48" t="s">
-        <v>159</v>
+        <v>81</v>
       </c>
       <c r="E48" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F48">
         <v>1</v>
@@ -2700,27 +1714,27 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>113</v>
-      </c>
-      <c r="D49" s="7" t="s">
-        <v>167</v>
+        <v>55</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>89</v>
       </c>
       <c r="E49" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F49">
         <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>119</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>179</v>
+      <c r="A50" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D50" s="7" t="s">
+        <v>101</v>
       </c>
       <c r="E50" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F50">
         <v>1</v>
@@ -2728,14 +1742,14 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="B51" s="4"/>
-      <c r="D51" s="8" t="s">
-        <v>182</v>
+      <c r="D51" s="7" t="s">
+        <v>104</v>
       </c>
       <c r="E51" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F51">
         <v>1</v>
@@ -2743,13 +1757,13 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>127</v>
-      </c>
-      <c r="D52" s="7" t="s">
-        <v>175</v>
+        <v>69</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>97</v>
       </c>
       <c r="E52" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F52">
         <v>1</v>
@@ -2757,23 +1771,23 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>117</v>
-      </c>
-      <c r="D53" s="7" t="s">
-        <v>181</v>
+        <v>59</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>103</v>
       </c>
       <c r="E53" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F53">
         <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="B55" s="9"/>
+      <c r="A55" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B55" s="8"/>
       <c r="F55" s="4"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -2781,58 +1795,58 @@
         <v>18</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>236</v>
+        <v>156</v>
       </c>
       <c r="E56" t="s">
-        <v>51</v>
-      </c>
-      <c r="F56" s="10">
+        <v>47</v>
+      </c>
+      <c r="F56" s="9">
         <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
-        <v>111</v>
+        <v>53</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="F57" s="10"/>
+        <v>158</v>
+      </c>
+      <c r="F57" s="9"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>126</v>
+        <v>68</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="F58" s="10"/>
+        <v>157</v>
+      </c>
+      <c r="F58" s="9"/>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>19</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>236</v>
+        <v>156</v>
       </c>
       <c r="E59" t="s">
-        <v>51</v>
-      </c>
-      <c r="F59" s="10">
+        <v>47</v>
+      </c>
+      <c r="F59" s="9">
         <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>114</v>
+        <v>56</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>236</v>
+        <v>156</v>
       </c>
       <c r="E60" t="s">
-        <v>51</v>
-      </c>
-      <c r="F60" s="10">
+        <v>47</v>
+      </c>
+      <c r="F60" s="9">
         <v>0</v>
       </c>
     </row>
@@ -2843,271 +1857,286 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>211</v>
+        <v>132</v>
       </c>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
       <c r="D62" s="1"/>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
-      <c r="G62" s="13"/>
+      <c r="G62" s="12"/>
       <c r="H62" s="1"/>
       <c r="I62" s="1"/>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E63" s="10" t="s">
-        <v>210</v>
+      <c r="E63" s="9" t="s">
+        <v>131</v>
       </c>
       <c r="F63" t="s">
-        <v>232</v>
-      </c>
-      <c r="G63" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="H63" s="10" t="s">
-        <v>222</v>
+        <v>153</v>
+      </c>
+      <c r="G63" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="H63" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="I63" s="9" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E64" s="10" t="s">
-        <v>206</v>
+      <c r="E64" s="9" t="s">
+        <v>127</v>
       </c>
       <c r="F64" t="s">
-        <v>232</v>
-      </c>
-      <c r="G64" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="H64" s="10" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="65" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E65" s="10" t="s">
-        <v>207</v>
+        <v>153</v>
+      </c>
+      <c r="G64" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="H64" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="I64" s="9" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="65" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E65" s="9" t="s">
+        <v>128</v>
       </c>
       <c r="F65" t="s">
-        <v>232</v>
-      </c>
-      <c r="G65" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="H65" s="10" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="66" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E66" s="10" t="s">
-        <v>212</v>
+        <v>153</v>
+      </c>
+      <c r="G65" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="H65" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="I65" s="9" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="66" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E66" s="9" t="s">
+        <v>133</v>
       </c>
       <c r="F66" t="s">
-        <v>232</v>
-      </c>
-      <c r="G66" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="H66" s="10" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="67" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E67" s="10" t="s">
-        <v>213</v>
+        <v>153</v>
+      </c>
+      <c r="G66" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="H66" s="9" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="67" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E67" s="9" t="s">
+        <v>134</v>
       </c>
       <c r="F67" t="s">
-        <v>232</v>
-      </c>
-      <c r="G67" s="10" t="s">
-        <v>220</v>
-      </c>
-      <c r="H67" s="10" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="68" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E68" s="10" t="s">
-        <v>214</v>
+        <v>153</v>
+      </c>
+      <c r="G67" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="H67" s="9" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="68" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E68" s="9" t="s">
+        <v>135</v>
       </c>
       <c r="F68" t="s">
-        <v>232</v>
-      </c>
-      <c r="G68" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="H68" s="10" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="69" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E69" s="10" t="s">
-        <v>215</v>
+        <v>153</v>
+      </c>
+      <c r="G68" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="H68" s="9" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="69" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E69" s="9" t="s">
+        <v>136</v>
       </c>
       <c r="F69" t="s">
-        <v>232</v>
-      </c>
-      <c r="G69" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="H69" s="10" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="70" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E70" s="10" t="s">
-        <v>216</v>
+        <v>153</v>
+      </c>
+      <c r="G69" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="H69" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="I69" s="9" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="70" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E70" s="9" t="s">
+        <v>137</v>
       </c>
       <c r="F70" t="s">
-        <v>232</v>
-      </c>
-      <c r="G70" s="10" t="s">
-        <v>220</v>
-      </c>
-      <c r="H70" s="10" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="71" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E71" s="10" t="s">
-        <v>217</v>
+        <v>153</v>
+      </c>
+      <c r="G70" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="H70" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="71" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E71" s="9" t="s">
+        <v>138</v>
       </c>
       <c r="F71" t="s">
-        <v>232</v>
-      </c>
-      <c r="G71" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="H71" s="10" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="72" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E72" s="10" t="s">
-        <v>218</v>
+        <v>153</v>
+      </c>
+      <c r="G71" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="H71" s="9" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="72" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E72" s="9" t="s">
+        <v>139</v>
       </c>
       <c r="F72" t="s">
-        <v>232</v>
-      </c>
-      <c r="G72" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="H72" s="10" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="73" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E73" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="F73" s="6">
+        <v>153</v>
+      </c>
+      <c r="G72" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="H72" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="I72" s="9" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="73" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E73" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="F73" s="5">
         <v>0</v>
       </c>
-      <c r="H73" s="6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="74" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E74" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="F74" s="6">
+      <c r="H73" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="74" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E74" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="F74" s="5">
         <v>0</v>
       </c>
-      <c r="G74" s="6"/>
-      <c r="H74" s="6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="75" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E75" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="F75" s="6">
+      <c r="G74" s="5"/>
+      <c r="H74" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E75" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="F75" s="5">
         <v>0</v>
       </c>
-      <c r="G75" s="6"/>
-      <c r="H75" s="6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="76" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E76" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="F76" s="6">
+      <c r="G75" s="5"/>
+      <c r="H75" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="76" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E76" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="F76" s="5">
         <v>0</v>
       </c>
-      <c r="H76" s="6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="77" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E77" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="F77" s="6">
+      <c r="H76" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="77" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E77" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F77" s="5">
         <v>0</v>
       </c>
-      <c r="H77" s="6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="78" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E78" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="F78" s="6">
+      <c r="H77" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="78" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E78" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F78" s="5">
         <v>0</v>
       </c>
-      <c r="H78" s="6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="79" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E79" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="F79" s="6">
+      <c r="H78" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="79" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E79" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="F79" s="5">
         <v>0</v>
       </c>
-      <c r="G79" s="6"/>
-      <c r="H79" s="6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="80" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E80" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="F80" s="6">
+      <c r="G79" s="5"/>
+      <c r="H79" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="80" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E80" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F80" s="5">
         <v>0</v>
       </c>
-      <c r="G80" s="6"/>
-      <c r="H80" s="6" t="s">
-        <v>151</v>
+      <c r="G80" s="5"/>
+      <c r="H80" s="5" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E81" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="F81" s="6">
+      <c r="E81" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="F81" s="5">
         <v>0</v>
       </c>
-      <c r="G81" s="6"/>
-      <c r="H81" s="6" t="s">
-        <v>151</v>
+      <c r="G81" s="5"/>
+      <c r="H81" s="5" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E82" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="F82" s="6">
+      <c r="E82" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="F82" s="5">
         <v>0</v>
       </c>
-      <c r="G82" s="6"/>
-      <c r="H82" s="6" t="s">
-        <v>151</v>
+      <c r="G82" s="5"/>
+      <c r="H82" s="5" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -3115,7 +2144,7 @@
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>184</v>
+        <v>106</v>
       </c>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
@@ -3123,118 +2152,118 @@
       <c r="E84" s="2"/>
       <c r="F84" s="2"/>
       <c r="G84" s="2" t="s">
-        <v>183</v>
+        <v>105</v>
       </c>
       <c r="H84" s="2"/>
       <c r="I84" s="2"/>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E85" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="F85" s="6">
+      <c r="E85" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="F85" s="5">
         <v>0</v>
       </c>
-      <c r="G85" s="6"/>
-      <c r="H85" s="6" t="s">
-        <v>151</v>
+      <c r="G85" s="5"/>
+      <c r="H85" s="5" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C86" t="s">
         <v>11</v>
       </c>
       <c r="D86" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E86" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F86">
         <v>210</v>
       </c>
       <c r="I86" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C87" t="s">
         <v>11</v>
       </c>
       <c r="D87" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E87" t="s">
-        <v>185</v>
-      </c>
-      <c r="F87" s="10">
+        <v>107</v>
+      </c>
+      <c r="F87" s="9">
         <v>235</v>
       </c>
       <c r="I87" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C88" t="s">
         <v>12</v>
       </c>
       <c r="D88" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E88" t="s">
-        <v>185</v>
-      </c>
-      <c r="F88" s="10">
+        <v>107</v>
+      </c>
+      <c r="F88" s="9">
         <v>230</v>
       </c>
       <c r="I88" t="s">
-        <v>187</v>
+        <v>109</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C89" t="s">
         <v>12</v>
       </c>
       <c r="D89" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E89" t="s">
-        <v>185</v>
-      </c>
-      <c r="F89" s="10">
+        <v>107</v>
+      </c>
+      <c r="F89" s="9">
         <v>230</v>
       </c>
       <c r="I89" t="s">
-        <v>187</v>
+        <v>109</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D90" t="s">
-        <v>153</v>
+        <v>75</v>
       </c>
       <c r="E90" t="s">
-        <v>185</v>
-      </c>
-      <c r="F90" s="10">
+        <v>107</v>
+      </c>
+      <c r="F90" s="9">
         <v>140</v>
       </c>
       <c r="I90" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -3242,16 +2271,16 @@
         <v>14</v>
       </c>
       <c r="D91" t="s">
-        <v>150</v>
+        <v>72</v>
       </c>
       <c r="E91" t="s">
-        <v>185</v>
-      </c>
-      <c r="F91" s="10">
+        <v>107</v>
+      </c>
+      <c r="F91" s="9">
         <v>180</v>
       </c>
       <c r="I91" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -3262,16 +2291,16 @@
         <v>11</v>
       </c>
       <c r="D92" t="s">
-        <v>150</v>
+        <v>72</v>
       </c>
       <c r="E92" t="s">
-        <v>185</v>
-      </c>
-      <c r="F92" s="10">
+        <v>107</v>
+      </c>
+      <c r="F92" s="9">
         <v>180</v>
       </c>
       <c r="I92" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -3282,16 +2311,16 @@
         <v>12</v>
       </c>
       <c r="D93" t="s">
-        <v>150</v>
+        <v>72</v>
       </c>
       <c r="E93" t="s">
-        <v>185</v>
-      </c>
-      <c r="F93" s="10">
+        <v>107</v>
+      </c>
+      <c r="F93" s="9">
         <v>210</v>
       </c>
       <c r="H93" t="s">
-        <v>192</v>
+        <v>114</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -3302,16 +2331,16 @@
         <v>12</v>
       </c>
       <c r="D94" t="s">
-        <v>150</v>
+        <v>72</v>
       </c>
       <c r="E94" t="s">
-        <v>185</v>
-      </c>
-      <c r="F94" s="10">
+        <v>107</v>
+      </c>
+      <c r="F94" s="9">
         <v>210</v>
       </c>
       <c r="I94" t="s">
-        <v>187</v>
+        <v>109</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -3322,16 +2351,16 @@
         <v>11</v>
       </c>
       <c r="D95" t="s">
-        <v>154</v>
+        <v>76</v>
       </c>
       <c r="E95" t="s">
-        <v>185</v>
-      </c>
-      <c r="F95" s="10">
+        <v>107</v>
+      </c>
+      <c r="F95" s="9">
         <v>190</v>
       </c>
       <c r="I95" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -3342,50 +2371,50 @@
         <v>12</v>
       </c>
       <c r="D96" t="s">
-        <v>154</v>
+        <v>76</v>
       </c>
       <c r="E96" t="s">
-        <v>185</v>
-      </c>
-      <c r="F96" s="10">
+        <v>107</v>
+      </c>
+      <c r="F96" s="9">
         <v>230</v>
       </c>
       <c r="I96" t="s">
-        <v>187</v>
+        <v>109</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D97" t="s">
-        <v>161</v>
+        <v>83</v>
       </c>
       <c r="E97" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F97">
         <v>180</v>
       </c>
       <c r="I97" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D98" t="s">
-        <v>161</v>
+        <v>83</v>
       </c>
       <c r="E98" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F98">
         <v>180</v>
       </c>
       <c r="H98" t="s">
-        <v>193</v>
+        <v>115</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
@@ -3396,14 +2425,14 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
-        <v>115</v>
+        <v>57</v>
       </c>
       <c r="B100" s="4"/>
       <c r="D100" s="4" t="s">
-        <v>154</v>
+        <v>76</v>
       </c>
       <c r="E100" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F100" s="4">
         <v>100</v>
@@ -3411,14 +2440,14 @@
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="4" t="s">
-        <v>115</v>
+        <v>57</v>
       </c>
       <c r="B101" s="4"/>
       <c r="D101" s="4" t="s">
-        <v>153</v>
+        <v>75</v>
       </c>
       <c r="E101" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F101" s="4">
         <v>100</v>
@@ -3432,19 +2461,19 @@
         <v>11</v>
       </c>
       <c r="D102" t="s">
-        <v>162</v>
+        <v>84</v>
       </c>
       <c r="E102" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F102">
         <v>20</v>
       </c>
       <c r="H102" t="s">
-        <v>189</v>
+        <v>111</v>
       </c>
       <c r="I102" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -3455,19 +2484,19 @@
         <v>12</v>
       </c>
       <c r="D103" t="s">
-        <v>162</v>
+        <v>84</v>
       </c>
       <c r="E103" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F103">
         <v>21</v>
       </c>
       <c r="H103" t="s">
-        <v>189</v>
+        <v>111</v>
       </c>
       <c r="I103" t="s">
-        <v>187</v>
+        <v>109</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -3484,16 +2513,16 @@
         <v>11</v>
       </c>
       <c r="D105" t="s">
-        <v>163</v>
+        <v>85</v>
       </c>
       <c r="E105" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F105">
         <v>9</v>
       </c>
       <c r="I105" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -3504,94 +2533,94 @@
         <v>12</v>
       </c>
       <c r="D106" t="s">
-        <v>163</v>
+        <v>85</v>
       </c>
       <c r="E106" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F106">
         <v>9.5</v>
       </c>
       <c r="I106" t="s">
-        <v>187</v>
+        <v>109</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="4" t="s">
-        <v>152</v>
+        <v>74</v>
       </c>
       <c r="B107" s="4"/>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>125</v>
+        <v>67</v>
       </c>
       <c r="C108" t="s">
         <v>11</v>
       </c>
       <c r="D108" t="s">
-        <v>160</v>
+        <v>82</v>
       </c>
       <c r="E108" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F108">
         <v>0.33</v>
       </c>
       <c r="I108" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>125</v>
+        <v>67</v>
       </c>
       <c r="C109" t="s">
         <v>12</v>
       </c>
       <c r="D109" t="s">
-        <v>160</v>
+        <v>82</v>
       </c>
       <c r="E109" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F109">
         <f>(5+0.4)/2</f>
         <v>2.7</v>
       </c>
       <c r="H109" t="s">
-        <v>188</v>
+        <v>110</v>
       </c>
       <c r="I109" t="s">
-        <v>187</v>
+        <v>109</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>124</v>
+        <v>66</v>
       </c>
       <c r="D110" t="s">
-        <v>160</v>
+        <v>82</v>
       </c>
       <c r="E110" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F110">
         <v>0.67</v>
       </c>
       <c r="I110" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>122</v>
+        <v>64</v>
       </c>
       <c r="D111" t="s">
-        <v>156</v>
+        <v>78</v>
       </c>
       <c r="E111" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F111">
         <f>900+1800</f>
@@ -3600,31 +2629,31 @@
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>121</v>
+        <v>63</v>
       </c>
       <c r="D112" t="s">
-        <v>155</v>
+        <v>77</v>
       </c>
       <c r="E112" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F112">
         <v>2000</v>
       </c>
       <c r="H112" t="s">
-        <v>190</v>
-      </c>
-      <c r="I112" s="11" t="s">
-        <v>191</v>
+        <v>112</v>
+      </c>
+      <c r="I112" s="10" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B113" s="4"/>
       <c r="H113" s="4" t="s">
-        <v>194</v>
+        <v>116</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -3633,10 +2662,10 @@
       </c>
       <c r="B114" s="4"/>
       <c r="D114" t="s">
-        <v>173</v>
+        <v>95</v>
       </c>
       <c r="E114" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F114" s="4">
         <v>5</v>
@@ -3650,13 +2679,13 @@
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
-        <v>111</v>
+        <v>53</v>
       </c>
       <c r="B116" s="4"/>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" s="4" t="s">
-        <v>126</v>
+        <v>68</v>
       </c>
       <c r="B117" s="4"/>
     </row>
@@ -3667,54 +2696,54 @@
       <c r="B118" s="4"/>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A119" s="10" t="s">
+      <c r="A119" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B119" s="4"/>
       <c r="D119" t="s">
-        <v>173</v>
+        <v>95</v>
       </c>
       <c r="E119" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F119">
         <v>7</v>
       </c>
       <c r="H119" s="4" t="s">
-        <v>195</v>
+        <v>117</v>
       </c>
       <c r="I119" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A120" s="10" t="s">
+      <c r="A120" s="9" t="s">
         <v>23</v>
       </c>
       <c r="B120" s="4"/>
       <c r="D120" t="s">
-        <v>173</v>
+        <v>95</v>
       </c>
       <c r="E120" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
       <c r="F120">
         <v>4</v>
       </c>
       <c r="H120" s="4" t="s">
-        <v>197</v>
+        <v>119</v>
       </c>
       <c r="I120" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="4" t="s">
-        <v>114</v>
+        <v>56</v>
       </c>
       <c r="B121" s="4"/>
       <c r="H121" s="4" t="s">
-        <v>196</v>
+        <v>118</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -3736,155 +2765,194 @@
       <c r="B124" s="4"/>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A125" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B125" s="4"/>
+      <c r="A125" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B125" s="9"/>
+      <c r="C125" s="9"/>
+      <c r="D125" s="9"/>
+      <c r="E125" s="9"/>
+      <c r="F125" s="9">
+        <v>0</v>
+      </c>
+      <c r="H125" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A126" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B126" s="4"/>
+      <c r="A126" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B126" s="9"/>
+      <c r="C126" s="9"/>
+      <c r="D126" s="9"/>
+      <c r="E126" s="9"/>
+      <c r="F126" s="9">
+        <v>0</v>
+      </c>
+      <c r="H126" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="4" t="s">
-        <v>116</v>
+        <v>58</v>
       </c>
       <c r="B127" s="4"/>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
-        <v>108</v>
+        <v>50</v>
       </c>
       <c r="B128" s="4"/>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" s="4" t="s">
-        <v>118</v>
+        <v>60</v>
       </c>
       <c r="B129" s="4"/>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B130" s="4"/>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B131" s="4"/>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>109</v>
+        <v>51</v>
       </c>
       <c r="B132" s="4"/>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" s="4" t="s">
-        <v>123</v>
+        <v>65</v>
       </c>
       <c r="B133" s="4"/>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" s="4" t="s">
         <v>20</v>
       </c>
       <c r="B134" s="4"/>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B135" s="4"/>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B136" s="4"/>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" s="4" t="s">
-        <v>110</v>
+        <v>52</v>
       </c>
       <c r="B137" s="4"/>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" s="4" t="s">
         <v>28</v>
       </c>
       <c r="B138" s="4"/>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B139" s="4"/>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" s="4" t="s">
-        <v>120</v>
+        <v>62</v>
       </c>
       <c r="B140" s="4"/>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" s="4" t="s">
         <v>30</v>
       </c>
       <c r="B141" s="4"/>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="B142" s="4"/>
-    </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G142" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" s="4" t="s">
-        <v>158</v>
+        <v>80</v>
       </c>
       <c r="B143" s="4"/>
-    </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G143" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" s="4" t="s">
-        <v>113</v>
+        <v>55</v>
       </c>
       <c r="B144" s="4"/>
+      <c r="G144" s="4" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" s="4" t="s">
-        <v>119</v>
+        <v>61</v>
       </c>
       <c r="B145" s="4"/>
+      <c r="G145" s="4" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" s="4" t="s">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="B146" s="4"/>
+      <c r="G146" s="4" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" s="4" t="s">
-        <v>127</v>
+        <v>69</v>
       </c>
       <c r="B147" s="4"/>
+      <c r="G147" s="4" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" s="4" t="s">
-        <v>117</v>
+        <v>59</v>
       </c>
       <c r="B148" s="4"/>
+      <c r="G148" s="4" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="F149" s="4"/>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
-        <v>198</v>
+        <v>120</v>
       </c>
       <c r="B150" s="1"/>
       <c r="C150" s="1"/>
@@ -3897,68 +2965,68 @@
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B151" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E151" t="s">
-        <v>200</v>
-      </c>
-      <c r="F151" s="12">
+        <v>122</v>
+      </c>
+      <c r="F151" s="11">
         <f>1/7*100</f>
         <v>14.285714285714285</v>
       </c>
       <c r="G151" t="s">
-        <v>201</v>
+        <v>123</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B152" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="C152" t="s">
         <v>12</v>
       </c>
       <c r="E152" t="s">
-        <v>200</v>
+        <v>122</v>
       </c>
       <c r="F152" s="4">
         <f>1/8*100</f>
         <v>12.5</v>
       </c>
       <c r="G152" t="s">
-        <v>201</v>
+        <v>123</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B153" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="E153" t="s">
-        <v>200</v>
-      </c>
-      <c r="F153" s="12">
+        <v>122</v>
+      </c>
+      <c r="F153" s="11">
         <f>1/6*100</f>
         <v>16.666666666666664</v>
       </c>
       <c r="G153" t="s">
-        <v>201</v>
+        <v>123</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B154" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C154" t="s">
         <v>12</v>
       </c>
       <c r="E154" t="s">
-        <v>200</v>
-      </c>
-      <c r="F154" s="12">
+        <v>122</v>
+      </c>
+      <c r="F154" s="11">
         <f>1/10*100</f>
         <v>10</v>
       </c>
       <c r="G154" t="s">
-        <v>201</v>
+        <v>123</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -3966,7 +3034,7 @@
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
-        <v>46</v>
+        <v>169</v>
       </c>
       <c r="B156" s="1"/>
       <c r="C156" s="1"/>
@@ -3974,23 +3042,21 @@
       <c r="E156" s="2"/>
       <c r="F156" s="2"/>
       <c r="G156" s="2" t="s">
-        <v>107</v>
+        <v>167</v>
       </c>
       <c r="H156" s="2"/>
-      <c r="I156" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="I156" s="2"/>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E157" s="6" t="s">
+      <c r="E157" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F157" s="6">
+      <c r="F157" s="5">
         <v>0</v>
       </c>
-      <c r="G157" s="6"/>
-      <c r="H157" s="6" t="s">
-        <v>151</v>
+      <c r="G157" s="5"/>
+      <c r="H157" s="5" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
@@ -3998,15 +3064,18 @@
         <v>7</v>
       </c>
       <c r="F158" t="s">
-        <v>233</v>
+        <v>154</v>
       </c>
       <c r="H158" t="s">
-        <v>202</v>
+        <v>124</v>
+      </c>
+      <c r="I158" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
-        <v>204</v>
+        <v>126</v>
       </c>
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
@@ -4022,13 +3091,13 @@
         <v>10</v>
       </c>
       <c r="E162" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F162">
         <v>1508</v>
       </c>
       <c r="G162" t="s">
-        <v>205</v>
+        <v>168</v>
       </c>
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.25">
@@ -4036,7 +3105,7 @@
         <v>13</v>
       </c>
       <c r="E163" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F163">
         <v>980</v>
@@ -4047,7 +3116,7 @@
         <v>14</v>
       </c>
       <c r="E164" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F164">
         <v>1212</v>
@@ -4055,10 +3124,10 @@
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>152</v>
+        <v>74</v>
       </c>
       <c r="E165" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F165">
         <v>1779</v>
@@ -4069,7 +3138,7 @@
         <v>15</v>
       </c>
       <c r="E166" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F166">
         <v>1092</v>
@@ -4080,7 +3149,7 @@
         <v>16</v>
       </c>
       <c r="E167" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F167">
         <v>1016</v>
@@ -4088,10 +3157,10 @@
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>108</v>
+        <v>50</v>
       </c>
       <c r="E168" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F168">
         <v>1016</v>
@@ -4102,7 +3171,7 @@
         <v>17</v>
       </c>
       <c r="E169" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F169">
         <v>649</v>
@@ -4110,10 +3179,10 @@
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>109</v>
+        <v>51</v>
       </c>
       <c r="E170" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F170">
         <v>1185</v>
@@ -4121,10 +3190,10 @@
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>158</v>
+        <v>80</v>
       </c>
       <c r="E171" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F171">
         <v>1016</v>
@@ -4132,10 +3201,10 @@
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>110</v>
+        <v>52</v>
       </c>
       <c r="E172" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F172">
         <v>945</v>
@@ -4143,10 +3212,10 @@
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>111</v>
+        <v>53</v>
       </c>
       <c r="E173" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F173">
         <v>945</v>
@@ -4157,7 +3226,7 @@
         <v>18</v>
       </c>
       <c r="E174" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F174">
         <v>628</v>
@@ -4168,7 +3237,7 @@
         <v>19</v>
       </c>
       <c r="E175" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F175">
         <v>1016</v>
@@ -4179,7 +3248,7 @@
         <v>20</v>
       </c>
       <c r="E176" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F176">
         <v>1185</v>
@@ -4187,10 +3256,10 @@
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="E177" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F177">
         <v>1092</v>
@@ -4201,7 +3270,7 @@
         <v>21</v>
       </c>
       <c r="E178" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F178">
         <v>1016</v>
@@ -4209,10 +3278,10 @@
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>113</v>
+        <v>55</v>
       </c>
       <c r="E179" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F179">
         <v>1475</v>
@@ -4223,7 +3292,7 @@
         <v>22</v>
       </c>
       <c r="E180" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F180">
         <v>628</v>
@@ -4234,7 +3303,7 @@
         <v>23</v>
       </c>
       <c r="E181" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F181">
         <v>628</v>
@@ -4245,7 +3314,7 @@
         <v>24</v>
       </c>
       <c r="E182" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F182">
         <v>1074</v>
@@ -4253,10 +3322,10 @@
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>114</v>
+        <v>56</v>
       </c>
       <c r="E183" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F183">
         <v>628</v>
@@ -4267,7 +3336,7 @@
         <v>25</v>
       </c>
       <c r="E184" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F184">
         <v>1487</v>
@@ -4278,7 +3347,7 @@
         <v>26</v>
       </c>
       <c r="E185" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F185">
         <v>1487</v>
@@ -4286,10 +3355,10 @@
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>115</v>
+        <v>57</v>
       </c>
       <c r="E186" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F186">
         <v>649</v>
@@ -4300,7 +3369,7 @@
         <v>27</v>
       </c>
       <c r="E187" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F187">
         <v>980</v>
@@ -4308,10 +3377,10 @@
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>116</v>
+        <v>58</v>
       </c>
       <c r="E188" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F188">
         <v>1074</v>
@@ -4322,7 +3391,7 @@
         <v>28</v>
       </c>
       <c r="E189" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F189">
         <v>945</v>
@@ -4330,10 +3399,10 @@
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>117</v>
+        <v>59</v>
       </c>
       <c r="E190" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F190">
         <v>1016</v>
@@ -4344,7 +3413,7 @@
         <v>29</v>
       </c>
       <c r="E191" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F191">
         <v>767</v>
@@ -4355,7 +3424,7 @@
         <v>30</v>
       </c>
       <c r="E192" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F192">
         <v>1508</v>
@@ -4363,10 +3432,10 @@
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>118</v>
+        <v>60</v>
       </c>
       <c r="E193" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F193">
         <v>1016</v>
@@ -4377,7 +3446,7 @@
         <v>31</v>
       </c>
       <c r="E194" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F194">
         <v>1016</v>
@@ -4385,10 +3454,10 @@
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>119</v>
+        <v>61</v>
       </c>
       <c r="E195" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F195">
         <v>1185</v>
@@ -4396,10 +3465,10 @@
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>120</v>
+        <v>62</v>
       </c>
       <c r="E196" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F196">
         <v>1508</v>
@@ -4410,7 +3479,7 @@
         <v>32</v>
       </c>
       <c r="E197" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F197">
         <v>1212</v>
@@ -4421,7 +3490,7 @@
         <v>33</v>
       </c>
       <c r="E198" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F198">
         <v>1569</v>
@@ -4429,10 +3498,10 @@
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>121</v>
+        <v>63</v>
       </c>
       <c r="E199" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F199">
         <v>1569</v>
@@ -4440,10 +3509,10 @@
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>122</v>
+        <v>64</v>
       </c>
       <c r="E200" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F200">
         <v>767</v>
@@ -4451,10 +3520,10 @@
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>123</v>
+        <v>65</v>
       </c>
       <c r="E201" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F201">
         <v>1185</v>
@@ -4462,10 +3531,10 @@
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>124</v>
+        <v>66</v>
       </c>
       <c r="E202" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F202">
         <v>1016</v>
@@ -4473,10 +3542,10 @@
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>125</v>
+        <v>67</v>
       </c>
       <c r="E203" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F203">
         <v>1212</v>
@@ -4484,10 +3553,10 @@
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E204" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F204">
         <v>1016</v>
@@ -4495,10 +3564,10 @@
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E205" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F205">
         <v>628</v>
@@ -4506,10 +3575,10 @@
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E206" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F206">
         <v>628</v>
@@ -4517,10 +3586,10 @@
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>126</v>
+        <v>68</v>
       </c>
       <c r="E207" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F207">
         <v>1225</v>
@@ -4528,10 +3597,10 @@
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E208" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F208">
         <v>1016</v>
@@ -4539,10 +3608,10 @@
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>127</v>
+        <v>69</v>
       </c>
       <c r="E209" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F209">
         <v>1016</v>
@@ -4550,10 +3619,10 @@
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E210" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F210">
         <v>1721</v>
@@ -4561,10 +3630,10 @@
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="E211" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F211">
         <v>1016</v>
@@ -4572,10 +3641,10 @@
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E212" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F212">
         <v>1212</v>
@@ -4583,10 +3652,10 @@
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E213" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F213">
         <v>1212</v>
@@ -4594,10 +3663,10 @@
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E214" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F214">
         <v>980</v>
@@ -4605,10 +3674,10 @@
     </row>
     <row r="215" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E215" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F215">
         <v>1016</v>
@@ -4627,38 +3696,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1.05</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Moved handling of pasture utilisation to CropProduction and updated feed losses
</commit_message>
<xml_diff>
--- a/data/prod_parameters/CropProduction.xlsx
+++ b/data/prod_parameters/CropProduction.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="174">
   <si>
     <t>f_crop</t>
   </si>
@@ -554,6 +554,18 @@
   </si>
   <si>
     <t>Yields</t>
+  </si>
+  <si>
+    <t>62.5% pasture utilisation</t>
+  </si>
+  <si>
+    <t>45% pasture utilisation. Should separate different types</t>
+  </si>
+  <si>
+    <t>Serina Ahlgren, Danira Behaderovic, Stefan Wirsenius, Annelie Carlsson, Anna Hessle, Per Toräng, Anett Seeman, Theo den Braver, Olle Kvarnbäck (2022) Miljöpåverkan av svensk nöt- och lammköttsproduktion</t>
+  </si>
+  <si>
+    <t>Ahlgren et al (2022)</t>
   </si>
 </sst>
 </file>
@@ -1230,7 +1242,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -1247,7 +1259,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>74</v>
       </c>
@@ -1261,7 +1273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>67</v>
       </c>
@@ -1275,7 +1287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>66</v>
       </c>
@@ -1289,7 +1301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>64</v>
       </c>
@@ -1303,7 +1315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>63</v>
       </c>
@@ -1317,7 +1329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>38</v>
       </c>
@@ -1331,7 +1343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -1345,7 +1357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -1363,7 +1375,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>23</v>
       </c>
@@ -1375,13 +1387,19 @@
         <v>47</v>
       </c>
       <c r="F26">
-        <v>1</v>
+        <v>0.625</v>
       </c>
       <c r="G26" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H26" t="s">
+        <v>170</v>
+      </c>
+      <c r="I26" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>26</v>
       </c>
@@ -1399,7 +1417,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>17</v>
       </c>
@@ -1417,7 +1435,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>29</v>
       </c>
@@ -1435,7 +1453,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>36</v>
       </c>
@@ -1447,13 +1465,19 @@
         <v>47</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>0.45</v>
       </c>
       <c r="G30" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H30" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="I30" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>35</v>
       </c>
@@ -1471,7 +1495,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>58</v>
       </c>
@@ -3698,7 +3722,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -3711,6 +3735,11 @@
         <v>163</v>
       </c>
     </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>172</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>